<commit_message>
fixed master template to include new fields in the plots. fixed fileio.
</commit_message>
<xml_diff>
--- a/inputs/slope/input_template_MASTER7.xlsx
+++ b/inputs/slope/input_template_MASTER7.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/inputs/slope/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/inputs/seep/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F27DC628-85FD-4448-9AF1-3D5AC21C40FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61E2C959-74FE-774E-8809-918B9D7782BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13400" yWindow="2880" windowWidth="37360" windowHeight="22440" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="31200" yWindow="2160" windowWidth="28700" windowHeight="22660" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="161">
   <si>
     <t>X</t>
   </si>
@@ -385,12 +385,6 @@
     <t>name</t>
   </si>
   <si>
-    <t>Clay</t>
-  </si>
-  <si>
-    <t>Sand</t>
-  </si>
-  <si>
     <t>Template version:</t>
   </si>
   <si>
@@ -504,12 +498,6 @@
     <t>seep bc</t>
   </si>
   <si>
-    <t>Shell</t>
-  </si>
-  <si>
-    <t>Core</t>
-  </si>
-  <si>
     <t>kr0</t>
   </si>
   <si>
@@ -619,6 +607,42 @@
   </si>
   <si>
     <t>Boundary condition set (b) is only used for a rapid drawdown analysis</t>
+  </si>
+  <si>
+    <t>Rip Rap 1</t>
+  </si>
+  <si>
+    <t>Shell 1</t>
+  </si>
+  <si>
+    <t>Rip Rap 2</t>
+  </si>
+  <si>
+    <t>Shell 2</t>
+  </si>
+  <si>
+    <t>Clay Core</t>
+  </si>
+  <si>
+    <t>Shell 3</t>
+  </si>
+  <si>
+    <t>Drain</t>
+  </si>
+  <si>
+    <t>Filter</t>
+  </si>
+  <si>
+    <t>Glacial Till 1</t>
+  </si>
+  <si>
+    <t>Glacial Till 2</t>
+  </si>
+  <si>
+    <t>Grouted Bedrock</t>
+  </si>
+  <si>
+    <t>Bedrock</t>
   </si>
 </sst>
 </file>
@@ -898,7 +922,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1033,11 +1057,6 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1154,16 +1173,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>150</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>270</c:v>
+                  <c:v>225</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>320</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>590</c:v>
+                  <c:v>240</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1175,16 +1191,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>227</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>317</c:v>
+                  <c:v>225</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>317</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>227</c:v>
+                  <c:v>230</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1244,13 +1257,7 @@
                   <c:v>240</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>280</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>310</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>350</c:v>
+                  <c:v>260</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1262,16 +1269,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>227</c:v>
+                  <c:v>230</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>307</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>307</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>227</c:v>
+                  <c:v>230</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1328,10 +1329,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>-150</c:v>
+                  <c:v>260</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>740</c:v>
+                  <c:v>316</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1343,10 +1344,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>227</c:v>
+                  <c:v>230</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>227</c:v>
+                  <c:v>202</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1403,10 +1404,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>-150</c:v>
+                  <c:v>153</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>740</c:v>
+                  <c:v>240</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1418,10 +1419,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>197</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>197</c:v>
+                  <c:v>229</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1477,6 +1478,15 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>210</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>240</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>250</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -1486,6 +1496,15 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>229</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>229</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1540,6 +1559,12 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>260</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>313</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -1549,6 +1574,12 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>229</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>202</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1609,6 +1640,21 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>255</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>260</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>260</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>316</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>320</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -1618,6 +1664,21 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>229</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>229</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>202</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>202</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>200</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1678,6 +1739,27 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>240</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>255</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>255</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>320</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>324</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -1687,6 +1769,27 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>190</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>202</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>229</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>229</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>198</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1747,6 +1850,15 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>210</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>215</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -1756,6 +1868,15 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>195</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1816,6 +1937,15 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>253</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>475</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -1825,6 +1955,15 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>198</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>198</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1873,24 +2012,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
-                <c:pt idx="0">
-                  <c:v>-150</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>277.5</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>315</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>343.5</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>590</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>740</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -1900,24 +2021,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
-                <c:pt idx="0">
-                  <c:v>302</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>302</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>275</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>240</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>227</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>227</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -2040,15 +2143,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>-150</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>225</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -2058,15 +2152,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>227</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>227</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>302</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -2346,15 +2431,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>-150</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>69</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -2364,15 +2440,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
-                <c:pt idx="0">
-                  <c:v>227</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>227</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>250</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -2635,24 +2702,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
-                <c:pt idx="0">
-                  <c:v>-150</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>251.5</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>315</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>347</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>590</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>740</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -2662,24 +2711,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
-                <c:pt idx="0">
-                  <c:v>250</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>250</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>242</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>233</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>227</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>227</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -2741,10 +2772,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>-150</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>150</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>225</c:v>
@@ -2759,13 +2790,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>227</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>227</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>302</c:v>
+                  <c:v>225</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2969,13 +3000,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
+                  <c:v>260</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>316</c:v>
+                </c:pt>
+                <c:pt idx="2">
                   <c:v>320</c:v>
                 </c:pt>
-                <c:pt idx="1">
-                  <c:v>590</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>740</c:v>
+                <c:pt idx="3">
+                  <c:v>324</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>475</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2987,13 +3024,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>317</c:v>
+                  <c:v>230</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>227</c:v>
+                  <c:v>202</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>227</c:v>
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>198</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>198</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3047,12 +3090,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
-                <c:pt idx="0">
-                  <c:v>39</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>109</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -3062,12 +3099,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
-                <c:pt idx="0">
-                  <c:v>240</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>240</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -3120,12 +3151,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
-                <c:pt idx="0">
-                  <c:v>84</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>154</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -3135,18 +3160,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>255</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>255</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>255</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>255</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -3199,12 +3212,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
-                <c:pt idx="0">
-                  <c:v>129</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>199</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -3214,12 +3221,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
-                <c:pt idx="0">
-                  <c:v>270</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>270</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -3272,12 +3273,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
-                <c:pt idx="0">
-                  <c:v>174</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>244</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -3287,12 +3282,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
-                <c:pt idx="0">
-                  <c:v>285</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>285</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -3348,12 +3337,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
-                <c:pt idx="0">
-                  <c:v>219</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>289</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -3363,12 +3346,6 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
-                <c:pt idx="0">
-                  <c:v>300</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>300</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -4321,6 +4298,711 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000014-6470-2847-A563-4EA99E47882D}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="45"/>
+          <c:order val="45"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>profile!$A$40</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Profile Line #11</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="70000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="70000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4">
+                    <a:lumMod val="70000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>profile!$A$42:$A$56</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>220</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>240</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>profile!$B$42:$B$56</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>190</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>190</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-E226-7045-8BAC-DB7411F222B8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="46"/>
+          <c:order val="46"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>profile!$D$40</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Profile Line #12</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="70000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="70000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent5">
+                    <a:lumMod val="70000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>profile!$D$42:$D$56</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>215</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>220</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>220</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>240</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>240</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>245</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>475</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>profile!$E$42:$E$56</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>190</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>140</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>140</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>190</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>190</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>195</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>195</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-E226-7045-8BAC-DB7411F222B8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="47"/>
+          <c:order val="47"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>profile!$G$40</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Profile Line #13</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="70000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="70000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent6">
+                    <a:lumMod val="70000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>profile!$G$42:$G$56</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>profile!$H$42:$H$56</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-E226-7045-8BAC-DB7411F222B8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="48"/>
+          <c:order val="48"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>profile!$J$40</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Profile Line #14</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="50000"/>
+                  <a:lumOff val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="50000"/>
+                  <a:lumOff val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="50000"/>
+                    <a:lumOff val="50000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>profile!$J$42:$J$56</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>profile!$K$42:$K$56</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-E226-7045-8BAC-DB7411F222B8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="49"/>
+          <c:order val="49"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>profile!$M$40</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Profile Line #15</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="50000"/>
+                  <a:lumOff val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="50000"/>
+                  <a:lumOff val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2">
+                    <a:lumMod val="50000"/>
+                    <a:lumOff val="50000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>profile!$M$42:$M$56</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>profile!$N$42:$N$56</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000005-E226-7045-8BAC-DB7411F222B8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="50"/>
+          <c:order val="50"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'seep bc'!$B$25:$C$25</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Specified Head #1(a)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="50000"/>
+                  <a:lumOff val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3">
+                  <a:lumMod val="50000"/>
+                  <a:lumOff val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3">
+                    <a:lumMod val="50000"/>
+                    <a:lumOff val="50000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'seep bc'!$B$28:$B$35</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'seep bc'!$C$28:$C$35</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000006-E226-7045-8BAC-DB7411F222B8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="51"/>
+          <c:order val="51"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'seep bc'!$E$25:$F$25</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Specified Head #2(b)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="50000"/>
+                  <a:lumOff val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="50000"/>
+                  <a:lumOff val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4">
+                    <a:lumMod val="50000"/>
+                    <a:lumOff val="50000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'seep bc'!$E$28:$E$35</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'seep bc'!$F$28:$F$35</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000007-E226-7045-8BAC-DB7411F222B8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="52"/>
+          <c:order val="52"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'seep bc'!$H$25:$I$25</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Specified Head #3(b)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="50000"/>
+                  <a:lumOff val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="50000"/>
+                  <a:lumOff val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent5">
+                    <a:lumMod val="50000"/>
+                    <a:lumOff val="50000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'seep bc'!$H$28:$H$35</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'seep bc'!$I$28:$I$35</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000008-E226-7045-8BAC-DB7411F222B8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="53"/>
+          <c:order val="53"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'seep bc'!$B$37:$C$37</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Exit Face (b)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="50000"/>
+                  <a:lumOff val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="50000"/>
+                  <a:lumOff val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent6">
+                    <a:lumMod val="50000"/>
+                    <a:lumOff val="50000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'seep bc'!$B$39:$B$46</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'seep bc'!$C$39:$C$46</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000009-E226-7045-8BAC-DB7411F222B8}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5105,13 +5787,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>589642</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>190500</xdr:rowOff>
+      <xdr:rowOff>190499</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>18142</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>166914</xdr:rowOff>
+      <xdr:colOff>9071</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>9070</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -5656,7 +6338,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="32" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="19" x14ac:dyDescent="0.25">
@@ -5666,7 +6348,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D5" s="39">
         <v>7</v>
@@ -5747,10 +6429,10 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B15" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D15" s="9"/>
     </row>
@@ -5828,34 +6510,34 @@
   <sheetData>
     <row r="2" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B2" s="45" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C2" s="45"/>
       <c r="E2" s="45" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="F2" s="45"/>
       <c r="H2" s="45" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="I2" s="45"/>
-      <c r="K2" s="52" t="s">
-        <v>147</v>
+      <c r="K2" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C3" s="31">
-        <v>302</v>
+        <v>225</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F3" s="31"/>
       <c r="H3" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="I3" s="31"/>
     </row>
@@ -5881,10 +6563,10 @@
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B5" s="3">
-        <v>-150</v>
+        <v>0</v>
       </c>
       <c r="C5" s="3">
-        <v>227</v>
+        <v>200</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -5893,10 +6575,10 @@
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B6" s="3">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="C6" s="3">
-        <v>227</v>
+        <v>200</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
@@ -5908,7 +6590,7 @@
         <v>225</v>
       </c>
       <c r="C7" s="3">
-        <v>302</v>
+        <v>225</v>
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
@@ -5957,7 +6639,7 @@
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B14" s="49" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C14" s="49"/>
     </row>
@@ -5971,35 +6653,43 @@
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B16" s="3">
-        <v>320</v>
+        <v>260</v>
       </c>
       <c r="C16" s="3">
-        <v>317</v>
+        <v>230</v>
       </c>
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B17" s="3">
-        <v>590</v>
-      </c>
-      <c r="C17" s="3">
-        <v>227</v>
+      <c r="B17" s="18">
+        <v>316</v>
+      </c>
+      <c r="C17" s="19">
+        <v>202</v>
       </c>
     </row>
     <row r="18" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B18" s="3">
-        <v>740</v>
+        <v>320</v>
       </c>
       <c r="C18" s="3">
-        <v>227</v>
+        <v>200</v>
       </c>
     </row>
     <row r="19" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
+      <c r="B19" s="3">
+        <v>324</v>
+      </c>
+      <c r="C19" s="3">
+        <v>198</v>
+      </c>
     </row>
     <row r="20" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
+      <c r="B20" s="3">
+        <v>475</v>
+      </c>
+      <c r="C20" s="3">
+        <v>198</v>
+      </c>
     </row>
     <row r="21" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B21" s="3"/>
@@ -6015,32 +6705,32 @@
     </row>
     <row r="25" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B25" s="45" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C25" s="45"/>
       <c r="E25" s="45" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="F25" s="45"/>
       <c r="H25" s="45" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="I25" s="45"/>
-      <c r="K25" s="52" t="s">
-        <v>152</v>
+      <c r="K25" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B26" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C26" s="31"/>
       <c r="E26" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F26" s="31"/>
       <c r="H26" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="I26" s="31"/>
     </row>
@@ -6130,7 +6820,7 @@
     </row>
     <row r="37" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B37" s="49" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C37" s="49"/>
     </row>
@@ -6223,7 +6913,7 @@
         <v>0</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
@@ -6282,93 +6972,93 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="B6" s="3">
-        <v>227</v>
+        <v>200</v>
       </c>
       <c r="D6" s="3">
         <v>240</v>
       </c>
       <c r="E6" s="3">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="G6" s="3">
-        <v>-150</v>
+        <v>260</v>
       </c>
       <c r="H6" s="3">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="J6" s="3">
-        <v>-150</v>
+        <v>153</v>
       </c>
       <c r="K6" s="3">
-        <v>197</v>
-      </c>
-      <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
+        <v>200</v>
+      </c>
+      <c r="M6" s="3">
+        <v>210</v>
+      </c>
+      <c r="N6" s="3">
+        <v>200</v>
+      </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
-        <v>270</v>
+        <v>225</v>
       </c>
       <c r="B7" s="3">
-        <v>317</v>
+        <v>225</v>
       </c>
       <c r="D7" s="3">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="E7" s="3">
-        <v>307</v>
+        <v>230</v>
       </c>
       <c r="G7" s="3">
-        <v>740</v>
+        <v>316</v>
       </c>
       <c r="H7" s="3">
-        <v>227</v>
+        <v>202</v>
       </c>
       <c r="J7" s="3">
-        <v>740</v>
+        <v>240</v>
       </c>
       <c r="K7" s="3">
-        <v>197</v>
-      </c>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
+        <v>229</v>
+      </c>
+      <c r="M7" s="3">
+        <v>240</v>
+      </c>
+      <c r="N7" s="3">
+        <v>229</v>
+      </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
-        <v>320</v>
+        <v>240</v>
       </c>
       <c r="B8" s="3">
-        <v>317</v>
-      </c>
-      <c r="D8" s="3">
-        <v>310</v>
-      </c>
-      <c r="E8" s="3">
-        <v>307</v>
-      </c>
+        <v>230</v>
+      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
+      <c r="M8" s="3">
+        <v>250</v>
+      </c>
+      <c r="N8" s="3">
+        <v>229</v>
+      </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A9" s="3">
-        <v>590</v>
-      </c>
-      <c r="B9" s="3">
-        <v>227</v>
-      </c>
-      <c r="D9" s="3">
-        <v>350</v>
-      </c>
-      <c r="E9" s="3">
-        <v>227</v>
-      </c>
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="J9" s="3"/>
@@ -6563,48 +7253,112 @@
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="17"/>
-      <c r="G24" s="16"/>
-      <c r="H24" s="17"/>
-      <c r="J24" s="16"/>
-      <c r="K24" s="17"/>
-      <c r="M24" s="16"/>
-      <c r="N24" s="17"/>
+      <c r="A24" s="3">
+        <v>260</v>
+      </c>
+      <c r="B24" s="3">
+        <v>229</v>
+      </c>
+      <c r="D24" s="16">
+        <v>255</v>
+      </c>
+      <c r="E24" s="17">
+        <v>229</v>
+      </c>
+      <c r="G24" s="16">
+        <v>240</v>
+      </c>
+      <c r="H24" s="17">
+        <v>190</v>
+      </c>
+      <c r="J24" s="16">
+        <v>0</v>
+      </c>
+      <c r="K24" s="17">
+        <v>200</v>
+      </c>
+      <c r="M24" s="16">
+        <v>250</v>
+      </c>
+      <c r="N24" s="17">
+        <v>195</v>
+      </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="19"/>
-      <c r="G25" s="18"/>
-      <c r="H25" s="19"/>
-      <c r="J25" s="18"/>
-      <c r="K25" s="19"/>
-      <c r="M25" s="18"/>
-      <c r="N25" s="19"/>
+      <c r="A25" s="3">
+        <v>313</v>
+      </c>
+      <c r="B25" s="3">
+        <v>202</v>
+      </c>
+      <c r="D25" s="18">
+        <v>260</v>
+      </c>
+      <c r="E25" s="19">
+        <v>229</v>
+      </c>
+      <c r="G25" s="18">
+        <v>250</v>
+      </c>
+      <c r="H25" s="19">
+        <v>202</v>
+      </c>
+      <c r="J25" s="18">
+        <v>210</v>
+      </c>
+      <c r="K25" s="19">
+        <v>200</v>
+      </c>
+      <c r="M25" s="18">
+        <v>253</v>
+      </c>
+      <c r="N25" s="19">
+        <v>198</v>
+      </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="19"/>
-      <c r="G26" s="18"/>
-      <c r="H26" s="19"/>
-      <c r="J26" s="18"/>
-      <c r="K26" s="19"/>
-      <c r="M26" s="18"/>
-      <c r="N26" s="19"/>
+      <c r="D26" s="18">
+        <v>260</v>
+      </c>
+      <c r="E26" s="19">
+        <v>202</v>
+      </c>
+      <c r="G26" s="18">
+        <v>250</v>
+      </c>
+      <c r="H26" s="19">
+        <v>229</v>
+      </c>
+      <c r="J26" s="18">
+        <v>215</v>
+      </c>
+      <c r="K26" s="19">
+        <v>195</v>
+      </c>
+      <c r="M26" s="18">
+        <v>475</v>
+      </c>
+      <c r="N26" s="19">
+        <v>198</v>
+      </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="19"/>
-      <c r="G27" s="18"/>
-      <c r="H27" s="19"/>
+      <c r="D27" s="18">
+        <v>316</v>
+      </c>
+      <c r="E27" s="19">
+        <v>202</v>
+      </c>
+      <c r="G27" s="16">
+        <v>255</v>
+      </c>
+      <c r="H27" s="17">
+        <v>229</v>
+      </c>
       <c r="J27" s="18"/>
       <c r="K27" s="19"/>
       <c r="M27" s="18"/>
@@ -6613,10 +7367,18 @@
     <row r="28" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="G28" s="3"/>
-      <c r="H28" s="3"/>
+      <c r="D28" s="3">
+        <v>320</v>
+      </c>
+      <c r="E28" s="3">
+        <v>200</v>
+      </c>
+      <c r="G28" s="3">
+        <v>255</v>
+      </c>
+      <c r="H28" s="3">
+        <v>200</v>
+      </c>
       <c r="J28" s="3"/>
       <c r="K28" s="3"/>
       <c r="M28" s="3"/>
@@ -6627,8 +7389,12 @@
       <c r="B29" s="3"/>
       <c r="D29" s="3"/>
       <c r="E29" s="3"/>
-      <c r="G29" s="3"/>
-      <c r="H29" s="3"/>
+      <c r="G29" s="3">
+        <v>320</v>
+      </c>
+      <c r="H29" s="3">
+        <v>200</v>
+      </c>
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
       <c r="M29" s="3"/>
@@ -6639,8 +7405,12 @@
       <c r="B30" s="3"/>
       <c r="D30" s="3"/>
       <c r="E30" s="3"/>
-      <c r="G30" s="3"/>
-      <c r="H30" s="3"/>
+      <c r="G30" s="3">
+        <v>324</v>
+      </c>
+      <c r="H30" s="3">
+        <v>198</v>
+      </c>
       <c r="J30" s="3"/>
       <c r="K30" s="3"/>
       <c r="M30" s="3"/>
@@ -6744,23 +7514,23 @@
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A40" s="42" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B40" s="42"/>
       <c r="D40" s="42" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="E40" s="42"/>
       <c r="G40" s="42" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="H40" s="42"/>
       <c r="J40" s="42" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="K40" s="42"/>
       <c r="M40" s="42" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="N40" s="42"/>
     </row>
@@ -6797,10 +7567,18 @@
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A42" s="3"/>
-      <c r="B42" s="3"/>
-      <c r="D42" s="16"/>
-      <c r="E42" s="17"/>
+      <c r="A42" s="3">
+        <v>220</v>
+      </c>
+      <c r="B42" s="3">
+        <v>190</v>
+      </c>
+      <c r="D42" s="16">
+        <v>0</v>
+      </c>
+      <c r="E42" s="17">
+        <v>195</v>
+      </c>
       <c r="G42" s="16"/>
       <c r="H42" s="17"/>
       <c r="J42" s="16"/>
@@ -6809,10 +7587,18 @@
       <c r="N42" s="17"/>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A43" s="3"/>
-      <c r="B43" s="3"/>
-      <c r="D43" s="18"/>
-      <c r="E43" s="19"/>
+      <c r="A43" s="3">
+        <v>240</v>
+      </c>
+      <c r="B43" s="3">
+        <v>190</v>
+      </c>
+      <c r="D43" s="18">
+        <v>215</v>
+      </c>
+      <c r="E43" s="19">
+        <v>195</v>
+      </c>
       <c r="G43" s="18"/>
       <c r="H43" s="19"/>
       <c r="J43" s="18"/>
@@ -6823,8 +7609,12 @@
     <row r="44" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
-      <c r="D44" s="18"/>
-      <c r="E44" s="19"/>
+      <c r="D44" s="18">
+        <v>220</v>
+      </c>
+      <c r="E44" s="19">
+        <v>190</v>
+      </c>
       <c r="G44" s="18"/>
       <c r="H44" s="19"/>
       <c r="J44" s="18"/>
@@ -6835,8 +7625,12 @@
     <row r="45" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A45" s="3"/>
       <c r="B45" s="3"/>
-      <c r="D45" s="18"/>
-      <c r="E45" s="19"/>
+      <c r="D45" s="18">
+        <v>220</v>
+      </c>
+      <c r="E45" s="19">
+        <v>140</v>
+      </c>
       <c r="G45" s="18"/>
       <c r="H45" s="19"/>
       <c r="J45" s="18"/>
@@ -6847,8 +7641,12 @@
     <row r="46" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A46" s="3"/>
       <c r="B46" s="3"/>
-      <c r="D46" s="3"/>
-      <c r="E46" s="3"/>
+      <c r="D46" s="3">
+        <v>240</v>
+      </c>
+      <c r="E46" s="3">
+        <v>140</v>
+      </c>
       <c r="G46" s="3"/>
       <c r="H46" s="3"/>
       <c r="J46" s="3"/>
@@ -6859,8 +7657,12 @@
     <row r="47" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A47" s="3"/>
       <c r="B47" s="3"/>
-      <c r="D47" s="3"/>
-      <c r="E47" s="3"/>
+      <c r="D47" s="3">
+        <v>240</v>
+      </c>
+      <c r="E47" s="3">
+        <v>190</v>
+      </c>
       <c r="G47" s="3"/>
       <c r="H47" s="3"/>
       <c r="J47" s="3"/>
@@ -6871,8 +7673,12 @@
     <row r="48" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A48" s="3"/>
       <c r="B48" s="3"/>
-      <c r="D48" s="3"/>
-      <c r="E48" s="3"/>
+      <c r="D48" s="3">
+        <v>245</v>
+      </c>
+      <c r="E48" s="3">
+        <v>190</v>
+      </c>
       <c r="G48" s="3"/>
       <c r="H48" s="3"/>
       <c r="J48" s="3"/>
@@ -6883,8 +7689,12 @@
     <row r="49" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A49" s="3"/>
       <c r="B49" s="3"/>
-      <c r="D49" s="3"/>
-      <c r="E49" s="3"/>
+      <c r="D49" s="3">
+        <v>250</v>
+      </c>
+      <c r="E49" s="3">
+        <v>195</v>
+      </c>
       <c r="G49" s="3"/>
       <c r="H49" s="3"/>
       <c r="J49" s="3"/>
@@ -6895,8 +7705,12 @@
     <row r="50" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A50" s="3"/>
       <c r="B50" s="3"/>
-      <c r="D50" s="3"/>
-      <c r="E50" s="3"/>
+      <c r="D50" s="3">
+        <v>475</v>
+      </c>
+      <c r="E50" s="3">
+        <v>195</v>
+      </c>
       <c r="G50" s="3"/>
       <c r="H50" s="3"/>
       <c r="J50" s="3"/>
@@ -7005,8 +7819,9 @@
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.33203125" style="1" customWidth="1"/>
-    <col min="3" max="9" width="8.5" style="1" customWidth="1"/>
-    <col min="10" max="13" width="8.5" customWidth="1"/>
+    <col min="3" max="9" width="8.5" style="1" hidden="1" customWidth="1"/>
+    <col min="10" max="13" width="8.5" hidden="1" customWidth="1"/>
+    <col min="14" max="17" width="0" hidden="1" customWidth="1"/>
     <col min="23" max="23" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
@@ -7037,14 +7852,14 @@
       <c r="P2" s="43"/>
       <c r="Q2" s="43"/>
       <c r="R2" s="43" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="S2" s="43"/>
       <c r="T2" s="43"/>
       <c r="U2" s="43"/>
       <c r="V2" s="43"/>
       <c r="W2" s="43" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="X2" s="43"/>
     </row>
@@ -7074,13 +7889,13 @@
         <v>73</v>
       </c>
       <c r="I3" s="21" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="J3" s="29" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="K3" s="21" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="L3" s="22" t="s">
         <v>54</v>
@@ -7095,31 +7910,31 @@
         <v>75</v>
       </c>
       <c r="P3" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="Q3" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="R3" s="28" t="s">
+        <v>104</v>
+      </c>
+      <c r="S3" s="28" t="s">
+        <v>105</v>
+      </c>
+      <c r="T3" s="28" t="s">
         <v>106</v>
       </c>
-      <c r="S3" s="28" t="s">
-        <v>107</v>
-      </c>
-      <c r="T3" s="28" t="s">
-        <v>108</v>
-      </c>
       <c r="U3" s="28" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="V3" s="28" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="W3" s="33" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="X3" s="34" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.2">
@@ -7127,39 +7942,29 @@
         <v>1</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="C4" s="3">
-        <v>125</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E4" s="3">
-        <v>0</v>
-      </c>
-      <c r="F4" s="3">
-        <v>34</v>
-      </c>
-      <c r="G4" s="3">
-        <v>30</v>
-      </c>
-      <c r="H4" s="3">
-        <v>120</v>
-      </c>
+        <v>149</v>
+      </c>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
-      <c r="K4" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="K4" s="3"/>
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
+      <c r="R4" s="3">
+        <v>100000</v>
+      </c>
+      <c r="S4" s="3">
+        <v>100000</v>
+      </c>
       <c r="T4" s="3"/>
       <c r="U4" s="3"/>
       <c r="V4" s="3"/>
@@ -7171,39 +7976,29 @@
         <v>2</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="C5" s="3">
-        <v>122</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E5" s="3">
-        <v>100</v>
-      </c>
-      <c r="F5" s="3">
-        <v>26</v>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
-      <c r="I5" s="3">
-        <v>300</v>
-      </c>
-      <c r="J5" s="3">
-        <v>20</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
       <c r="O5" s="3"/>
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
-      <c r="R5" s="3"/>
-      <c r="S5" s="3"/>
+      <c r="R5" s="3">
+        <v>250</v>
+      </c>
+      <c r="S5" s="3">
+        <v>50</v>
+      </c>
       <c r="T5" s="3"/>
       <c r="U5" s="3"/>
       <c r="V5" s="3"/>
@@ -7215,39 +8010,29 @@
         <v>3</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C6" s="3">
-        <v>123</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E6" s="3">
-        <v>0</v>
-      </c>
-      <c r="F6" s="3">
-        <v>24</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
-      <c r="I6" s="3">
-        <v>100</v>
-      </c>
-      <c r="J6" s="3">
-        <v>19</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
       <c r="O6" s="3"/>
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
-      <c r="R6" s="3"/>
-      <c r="S6" s="3"/>
+      <c r="R6" s="3">
+        <v>100000</v>
+      </c>
+      <c r="S6" s="3">
+        <v>100000</v>
+      </c>
       <c r="T6" s="3"/>
       <c r="U6" s="3"/>
       <c r="V6" s="3"/>
@@ -7259,35 +8044,29 @@
         <v>4</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="C7" s="3">
-        <v>127</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E7" s="3">
-        <v>0</v>
-      </c>
-      <c r="F7" s="3">
-        <v>32</v>
-      </c>
+        <v>152</v>
+      </c>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
-      <c r="K7" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="K7" s="3"/>
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
       <c r="N7" s="3"/>
       <c r="O7" s="3"/>
       <c r="P7" s="3"/>
       <c r="Q7" s="3"/>
-      <c r="R7" s="3"/>
-      <c r="S7" s="3"/>
+      <c r="R7" s="3">
+        <v>250</v>
+      </c>
+      <c r="S7" s="3">
+        <v>50</v>
+      </c>
       <c r="T7" s="3"/>
       <c r="U7" s="3"/>
       <c r="V7" s="3"/>
@@ -7298,7 +8077,9 @@
       <c r="A8" s="3">
         <v>5</v>
       </c>
-      <c r="B8" s="3"/>
+      <c r="B8" s="3" t="s">
+        <v>153</v>
+      </c>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
@@ -7314,8 +8095,12 @@
       <c r="O8" s="3"/>
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
-      <c r="R8" s="3"/>
-      <c r="S8" s="3"/>
+      <c r="R8" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="S8" s="3">
+        <v>0.1</v>
+      </c>
       <c r="T8" s="3"/>
       <c r="U8" s="3"/>
       <c r="V8" s="3"/>
@@ -7326,7 +8111,9 @@
       <c r="A9" s="3">
         <v>6</v>
       </c>
-      <c r="B9" s="3"/>
+      <c r="B9" s="3" t="s">
+        <v>154</v>
+      </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -7342,8 +8129,12 @@
       <c r="O9" s="3"/>
       <c r="P9" s="3"/>
       <c r="Q9" s="3"/>
-      <c r="R9" s="3"/>
-      <c r="S9" s="3"/>
+      <c r="R9" s="3">
+        <v>250</v>
+      </c>
+      <c r="S9" s="3">
+        <v>50</v>
+      </c>
       <c r="T9" s="3"/>
       <c r="U9" s="3"/>
       <c r="V9" s="3"/>
@@ -7354,7 +8145,9 @@
       <c r="A10" s="3">
         <v>7</v>
       </c>
-      <c r="B10" s="3"/>
+      <c r="B10" s="3" t="s">
+        <v>155</v>
+      </c>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
@@ -7370,8 +8163,12 @@
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
       <c r="Q10" s="3"/>
-      <c r="R10" s="3"/>
-      <c r="S10" s="3"/>
+      <c r="R10" s="3">
+        <v>10000</v>
+      </c>
+      <c r="S10" s="3">
+        <v>10000</v>
+      </c>
       <c r="T10" s="3"/>
       <c r="U10" s="3"/>
       <c r="V10" s="3"/>
@@ -7382,7 +8179,9 @@
       <c r="A11" s="3">
         <v>8</v>
       </c>
-      <c r="B11" s="3"/>
+      <c r="B11" s="3" t="s">
+        <v>156</v>
+      </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
@@ -7398,8 +8197,12 @@
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
       <c r="Q11" s="3"/>
-      <c r="R11" s="3"/>
-      <c r="S11" s="3"/>
+      <c r="R11" s="3">
+        <v>1000</v>
+      </c>
+      <c r="S11" s="3">
+        <v>1000</v>
+      </c>
       <c r="T11" s="3"/>
       <c r="U11" s="3"/>
       <c r="V11" s="3"/>
@@ -7410,7 +8213,9 @@
       <c r="A12" s="3">
         <v>9</v>
       </c>
-      <c r="B12" s="3"/>
+      <c r="B12" s="3" t="s">
+        <v>157</v>
+      </c>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
@@ -7426,8 +8231,12 @@
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
       <c r="Q12" s="3"/>
-      <c r="R12" s="3"/>
-      <c r="S12" s="3"/>
+      <c r="R12" s="3">
+        <v>4000</v>
+      </c>
+      <c r="S12" s="3">
+        <v>2000</v>
+      </c>
       <c r="T12" s="3"/>
       <c r="U12" s="3"/>
       <c r="V12" s="3"/>
@@ -7438,7 +8247,9 @@
       <c r="A13" s="3">
         <v>10</v>
       </c>
-      <c r="B13" s="3"/>
+      <c r="B13" s="3" t="s">
+        <v>158</v>
+      </c>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
@@ -7454,8 +8265,12 @@
       <c r="O13" s="3"/>
       <c r="P13" s="3"/>
       <c r="Q13" s="3"/>
-      <c r="R13" s="3"/>
-      <c r="S13" s="3"/>
+      <c r="R13" s="3">
+        <v>4000</v>
+      </c>
+      <c r="S13" s="3">
+        <v>2000</v>
+      </c>
       <c r="T13" s="3"/>
       <c r="U13" s="3"/>
       <c r="V13" s="3"/>
@@ -7466,7 +8281,9 @@
       <c r="A14" s="3">
         <v>11</v>
       </c>
-      <c r="B14" s="3"/>
+      <c r="B14" s="3" t="s">
+        <v>159</v>
+      </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
@@ -7482,8 +8299,12 @@
       <c r="O14" s="3"/>
       <c r="P14" s="3"/>
       <c r="Q14" s="3"/>
-      <c r="R14" s="3"/>
-      <c r="S14" s="3"/>
+      <c r="R14" s="3">
+        <v>250</v>
+      </c>
+      <c r="S14" s="3">
+        <v>250</v>
+      </c>
       <c r="T14" s="3"/>
       <c r="U14" s="3"/>
       <c r="V14" s="3"/>
@@ -7494,7 +8315,9 @@
       <c r="A15" s="3">
         <v>12</v>
       </c>
-      <c r="B15" s="3"/>
+      <c r="B15" s="3" t="s">
+        <v>160</v>
+      </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
@@ -7510,8 +8333,12 @@
       <c r="O15" s="3"/>
       <c r="P15" s="3"/>
       <c r="Q15" s="3"/>
-      <c r="R15" s="3"/>
-      <c r="S15" s="3"/>
+      <c r="R15" s="3">
+        <v>2000</v>
+      </c>
+      <c r="S15" s="3">
+        <v>1000</v>
+      </c>
       <c r="T15" s="3"/>
       <c r="U15" s="3"/>
       <c r="V15" s="3"/>
@@ -7603,30 +8430,19 @@
       <c r="X18" s="3"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A19" s="50"/>
-      <c r="B19" s="50"/>
-      <c r="C19" s="50"/>
-      <c r="D19" s="50"/>
-      <c r="E19" s="50"/>
-      <c r="F19" s="50"/>
-      <c r="G19" s="50"/>
-      <c r="H19" s="50"/>
-      <c r="I19" s="50"/>
-      <c r="J19" s="50"/>
-      <c r="K19" s="50"/>
-      <c r="L19" s="50"/>
-      <c r="M19" s="50"/>
-      <c r="N19" s="50"/>
-      <c r="O19" s="50"/>
-      <c r="P19" s="50"/>
-      <c r="Q19" s="50"/>
-      <c r="R19" s="50"/>
-      <c r="S19" s="50"/>
-      <c r="T19" s="50"/>
-      <c r="U19" s="50"/>
-      <c r="V19" s="50"/>
-      <c r="W19" s="50"/>
-      <c r="X19" s="51"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
+      <c r="O19" s="1"/>
+      <c r="P19" s="1"/>
+      <c r="Q19" s="1"/>
+      <c r="R19" s="1"/>
+      <c r="S19" s="1"/>
+      <c r="T19" s="1"/>
+      <c r="U19" s="1"/>
+      <c r="V19" s="1"/>
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.2">
       <c r="C21" t="s">
@@ -7636,22 +8452,22 @@
       <c r="E21"/>
       <c r="F21"/>
       <c r="K21" s="6" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="W21" s="5"/>
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.2">
       <c r="C22" s="24" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D22"/>
       <c r="E22"/>
       <c r="F22"/>
       <c r="K22" s="14" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="L22" s="44" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="M22" s="44"/>
       <c r="N22" s="44"/>
@@ -7665,10 +8481,10 @@
       <c r="E23"/>
       <c r="F23"/>
       <c r="K23" s="14" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="L23" s="44" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="M23" s="44"/>
       <c r="N23" s="44"/>
@@ -7684,7 +8500,7 @@
       <c r="E24"/>
       <c r="F24"/>
       <c r="K24" s="14" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="L24" s="44"/>
       <c r="M24" s="44"/>
@@ -7721,7 +8537,7 @@
     </row>
     <row r="28" spans="1:24" x14ac:dyDescent="0.2">
       <c r="C28" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D28"/>
       <c r="E28"/>
@@ -7729,7 +8545,7 @@
     </row>
     <row r="29" spans="1:24" x14ac:dyDescent="0.2">
       <c r="C29" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D29" t="s">
         <v>60</v>
@@ -7749,10 +8565,10 @@
     </row>
     <row r="31" spans="1:24" x14ac:dyDescent="0.2">
       <c r="C31" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -7765,12 +8581,12 @@
     <mergeCell ref="L22:Q22"/>
     <mergeCell ref="L2:Q2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E4:F19 R19:V19 M4:N19">
+  <conditionalFormatting sqref="E4:F19 M4:N19 R19:V19">
     <cfRule type="expression" dxfId="3" priority="2">
       <formula>$D4="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O19:Q19 G19:J19 G4:H18 O4:O18">
+  <conditionalFormatting sqref="G4:H18 O4:O18 G19:J19 O19:Q19">
     <cfRule type="expression" dxfId="2" priority="9">
       <formula>$D4="mc"</formula>
     </cfRule>
@@ -7807,11 +8623,11 @@
   <sheetData>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="45" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B2" s="45"/>
       <c r="D2" s="46" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E2" s="46"/>
     </row>
@@ -7830,88 +8646,40 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="3">
-        <v>-150</v>
-      </c>
-      <c r="B4" s="3">
-        <v>302</v>
-      </c>
-      <c r="D4" s="3">
-        <v>-150</v>
-      </c>
-      <c r="E4" s="3">
-        <v>250</v>
-      </c>
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="3">
-        <v>277.5</v>
-      </c>
-      <c r="B5" s="3">
-        <v>302</v>
-      </c>
-      <c r="D5" s="3">
-        <v>251.5</v>
-      </c>
-      <c r="E5" s="3">
-        <v>250</v>
-      </c>
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="3">
-        <v>315</v>
-      </c>
-      <c r="B6" s="3">
-        <v>275</v>
-      </c>
-      <c r="D6" s="3">
-        <v>315</v>
-      </c>
-      <c r="E6" s="3">
-        <v>242</v>
-      </c>
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="3">
-        <v>343.5</v>
-      </c>
-      <c r="B7" s="3">
-        <v>240</v>
-      </c>
-      <c r="D7" s="3">
-        <v>347</v>
-      </c>
-      <c r="E7" s="3">
-        <v>233</v>
-      </c>
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="3">
-        <v>590</v>
-      </c>
-      <c r="B8" s="3">
-        <v>227</v>
-      </c>
-      <c r="D8" s="3">
-        <v>590</v>
-      </c>
-      <c r="E8" s="3">
-        <v>227</v>
-      </c>
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="3">
-        <v>740</v>
-      </c>
-      <c r="B9" s="3">
-        <v>227</v>
-      </c>
-      <c r="D9" s="3">
-        <v>740</v>
-      </c>
-      <c r="E9" s="3">
-        <v>227</v>
-      </c>
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="3"/>
@@ -7969,7 +8737,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="D20" s="25" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -8343,22 +9111,22 @@
   <sheetData>
     <row r="2" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B2" s="47" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C2" s="47"/>
       <c r="D2" s="47"/>
       <c r="F2" s="47" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="G2" s="47"/>
       <c r="H2" s="47"/>
       <c r="J2" s="47" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="K2" s="47"/>
       <c r="L2" s="47"/>
       <c r="N2" s="47" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="O2" s="47"/>
       <c r="P2" s="47"/>
@@ -8402,15 +9170,9 @@
       </c>
     </row>
     <row r="4" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B4" s="3">
-        <v>-150</v>
-      </c>
-      <c r="C4" s="3">
-        <v>227</v>
-      </c>
-      <c r="D4" s="3">
-        <v>4680</v>
-      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
@@ -8422,15 +9184,9 @@
       <c r="P4" s="3"/>
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B5" s="3">
-        <v>0</v>
-      </c>
-      <c r="C5" s="3">
-        <v>227</v>
-      </c>
-      <c r="D5" s="3">
-        <v>4680</v>
-      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
@@ -8442,15 +9198,9 @@
       <c r="P5" s="3"/>
     </row>
     <row r="6" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B6" s="3">
-        <v>225</v>
-      </c>
-      <c r="C6" s="3">
-        <v>302</v>
-      </c>
-      <c r="D6" s="3">
-        <v>0</v>
-      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
@@ -8561,22 +9311,22 @@
     </row>
     <row r="15" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B15" s="48" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C15" s="48"/>
       <c r="D15" s="48"/>
       <c r="F15" s="48" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G15" s="48"/>
       <c r="H15" s="48"/>
       <c r="J15" s="48" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="K15" s="48"/>
       <c r="L15" s="48"/>
       <c r="N15" s="48" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="O15" s="48"/>
       <c r="P15" s="48"/>
@@ -8620,16 +9370,9 @@
       </c>
     </row>
     <row r="17" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B17" s="3">
-        <v>-150</v>
-      </c>
-      <c r="C17" s="3">
-        <v>227</v>
-      </c>
-      <c r="D17" s="3">
-        <f>23*62.4</f>
-        <v>1435.2</v>
-      </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
@@ -8641,16 +9384,9 @@
       <c r="P17" s="3"/>
     </row>
     <row r="18" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B18" s="3">
-        <v>0</v>
-      </c>
-      <c r="C18" s="3">
-        <v>227</v>
-      </c>
-      <c r="D18" s="3">
-        <f>23*62.4</f>
-        <v>1435.2</v>
-      </c>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
@@ -8662,15 +9398,9 @@
       <c r="P18" s="3"/>
     </row>
     <row r="19" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B19" s="3">
-        <v>69</v>
-      </c>
-      <c r="C19" s="3">
-        <v>250</v>
-      </c>
-      <c r="D19" s="3">
-        <v>0</v>
-      </c>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
@@ -8781,12 +9511,12 @@
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B28" s="26" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B29" s="27" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -8818,64 +9548,48 @@
         <v>25</v>
       </c>
       <c r="B2" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="F2" s="36" t="s">
+        <v>129</v>
+      </c>
+      <c r="G2" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="H2" s="36" t="s">
+        <v>132</v>
+      </c>
+      <c r="I2" s="36" t="s">
+        <v>133</v>
+      </c>
+      <c r="J2" s="37" t="s">
+        <v>122</v>
+      </c>
+      <c r="K2" s="37" t="s">
         <v>128</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>129</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="F2" s="36" t="s">
-        <v>133</v>
-      </c>
-      <c r="G2" s="37" t="s">
-        <v>138</v>
-      </c>
-      <c r="H2" s="36" t="s">
-        <v>136</v>
-      </c>
-      <c r="I2" s="36" t="s">
-        <v>137</v>
-      </c>
-      <c r="J2" s="37" t="s">
-        <v>126</v>
-      </c>
-      <c r="K2" s="37" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="3">
-        <v>39</v>
-      </c>
-      <c r="C3" s="3">
-        <v>240</v>
-      </c>
-      <c r="D3" s="3">
-        <v>109</v>
-      </c>
-      <c r="E3" s="3">
-        <v>240</v>
-      </c>
-      <c r="F3" s="3">
-        <v>2000</v>
-      </c>
-      <c r="G3" s="3">
-        <v>1500</v>
-      </c>
-      <c r="H3" s="3">
-        <v>10</v>
-      </c>
-      <c r="I3" s="3">
-        <v>10</v>
-      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
     </row>
@@ -8883,30 +9597,14 @@
       <c r="A4" s="3">
         <v>2</v>
       </c>
-      <c r="B4" s="3">
-        <v>84</v>
-      </c>
-      <c r="C4" s="3">
-        <v>255</v>
-      </c>
-      <c r="D4" s="3">
-        <v>154</v>
-      </c>
-      <c r="E4" s="3">
-        <v>255</v>
-      </c>
-      <c r="F4" s="3">
-        <v>2000</v>
-      </c>
-      <c r="G4" s="3">
-        <v>1500</v>
-      </c>
-      <c r="H4" s="3">
-        <v>10</v>
-      </c>
-      <c r="I4" s="3">
-        <v>10</v>
-      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
     </row>
@@ -8914,30 +9612,14 @@
       <c r="A5" s="3">
         <v>3</v>
       </c>
-      <c r="B5" s="3">
-        <v>129</v>
-      </c>
-      <c r="C5" s="3">
-        <v>270</v>
-      </c>
-      <c r="D5" s="3">
-        <v>199</v>
-      </c>
-      <c r="E5" s="3">
-        <v>270</v>
-      </c>
-      <c r="F5" s="3">
-        <v>2000</v>
-      </c>
-      <c r="G5" s="3">
-        <v>1500</v>
-      </c>
-      <c r="H5" s="3">
-        <v>10</v>
-      </c>
-      <c r="I5" s="3">
-        <v>10</v>
-      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
@@ -8945,30 +9627,14 @@
       <c r="A6" s="3">
         <v>4</v>
       </c>
-      <c r="B6" s="3">
-        <v>174</v>
-      </c>
-      <c r="C6" s="3">
-        <v>285</v>
-      </c>
-      <c r="D6" s="3">
-        <v>244</v>
-      </c>
-      <c r="E6" s="3">
-        <v>285</v>
-      </c>
-      <c r="F6" s="3">
-        <v>2000</v>
-      </c>
-      <c r="G6" s="3">
-        <v>1500</v>
-      </c>
-      <c r="H6" s="3">
-        <v>10</v>
-      </c>
-      <c r="I6" s="3">
-        <v>10</v>
-      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
     </row>
@@ -8976,30 +9642,14 @@
       <c r="A7" s="3">
         <v>5</v>
       </c>
-      <c r="B7" s="3">
-        <v>219</v>
-      </c>
-      <c r="C7" s="3">
-        <v>300</v>
-      </c>
-      <c r="D7" s="3">
-        <v>289</v>
-      </c>
-      <c r="E7" s="3">
-        <v>300</v>
-      </c>
-      <c r="F7" s="3">
-        <v>2000</v>
-      </c>
-      <c r="G7" s="3">
-        <v>1500</v>
-      </c>
-      <c r="H7" s="3">
-        <v>10</v>
-      </c>
-      <c r="I7" s="3">
-        <v>10</v>
-      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
@@ -9231,7 +9881,7 @@
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="F24" s="35"/>
       <c r="G24" s="9" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="H24" s="9"/>
       <c r="I24" s="9"/>
@@ -9239,7 +9889,7 @@
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="F25" s="38"/>
       <c r="G25" s="9" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="H25" s="9"/>
       <c r="I25" s="9"/>

</xml_diff>